<commit_message>
Keep internal vendor output available and align rendered workbook rates
</commit_message>
<xml_diff>
--- a/opportunities/otf_rapid_response_2026/vendor_submission_20261011/examples/WORKBOOK-EXERCISE.xlsx
+++ b/opportunities/otf_rapid_response_2026/vendor_submission_20261011/examples/WORKBOOK-EXERCISE.xlsx
@@ -177,7 +177,9 @@
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="1" fillId="0" fontId="2" numFmtId="164" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
     <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>

</xml_diff>